<commit_message>
feat: update seeding process and add role management scripts for improved data handling
</commit_message>
<xml_diff>
--- a/sample-holidays-import-2025.xlsx
+++ b/sample-holidays-import-2025.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Holidays 2025" sheetId="1" r:id="rId1"/>
+    <sheet name="Sample Holidays" sheetId="1" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
@@ -397,10 +397,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:C6"/>
   <cols>
-    <col min="1" max="1" width="15.83203125" customWidth="1"/>
-    <col min="2" max="2" width="15.83203125" customWidth="1"/>
+    <col min="1" max="1" width="12.83203125" customWidth="1"/>
+    <col min="2" max="2" width="12.83203125" customWidth="1"/>
     <col min="3" max="3" width="30.83203125" customWidth="1"/>
   </cols>
   <sheetData>
@@ -420,7 +420,7 @@
         <v>01-Jan-2025</v>
       </c>
       <c r="B2" t="str">
-        <v>Monday</v>
+        <v>Wednesday</v>
       </c>
       <c r="C2" t="str">
         <v>New Year's Day</v>
@@ -439,62 +439,40 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>14-Feb-2025</v>
+        <v>15-Aug-2025</v>
       </c>
       <c r="B4" t="str">
         <v>Friday</v>
       </c>
       <c r="C4" t="str">
-        <v>Valentine's Day</v>
+        <v>Independence Day</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>08-Mar-2025</v>
+        <v>02-Oct-2025</v>
       </c>
       <c r="B5" t="str">
-        <v>Saturday</v>
+        <v>Thursday</v>
       </c>
       <c r="C5" t="str">
-        <v>International Women's Day</v>
+        <v>Gandhi Jayanti</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>15-Aug-2025</v>
+        <v>25-Dec-2025</v>
       </c>
       <c r="B6" t="str">
-        <v>Friday</v>
+        <v>Thursday</v>
       </c>
       <c r="C6" t="str">
-        <v>Independence Day</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>02-Oct-2025</v>
-      </c>
-      <c r="B7" t="str">
-        <v>Thursday</v>
-      </c>
-      <c r="C7" t="str">
-        <v>Gandhi Jayanti</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>25-Dec-2025</v>
-      </c>
-      <c r="B8" t="str">
-        <v>Thursday</v>
-      </c>
-      <c r="C8" t="str">
-        <v>Christmas Day</v>
+        <v>Christmas</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C6"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>